<commit_message>
chore(rename): correct sensivitiy -> sensitivity; update refs
</commit_message>
<xml_diff>
--- a/Distributions/sensitivity_run_results_25012026.xlsx
+++ b/Distributions/sensitivity_run_results_25012026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://esait-my.sharepoint.com/personal/ivo_ferreira_esa_int/Documents/NewAthenaE2EPSF_v3/Distributions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="133" documentId="8_{E1C7CD1F-9ABC-5249-9B87-D7756653E306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0F9AB2DB-75A2-4744-882C-BC8111469C36}"/>
+  <xr:revisionPtr revIDLastSave="150" documentId="8_{E1C7CD1F-9ABC-5249-9B87-D7756653E306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10D268E6-8F7F-D14F-BE36-E381604D2AD4}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="68800" windowHeight="26880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -2874,22 +2874,22 @@
     </pivotField>
     <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
       <items count="3">
-        <item h="1" x="0"/>
+        <item x="0"/>
+        <item h="1" x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisPage" showAll="0">
+      <items count="3">
         <item x="1"/>
+        <item x="0"/>
         <item t="default"/>
       </items>
     </pivotField>
     <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
       <items count="3">
-        <item x="1"/>
-        <item h="1" x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
-      <items count="3">
-        <item h="1" x="0"/>
-        <item x="1"/>
+        <item x="0"/>
+        <item h="1" x="1"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -4454,7 +4454,7 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
@@ -4462,7 +4462,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
@@ -4470,7 +4470,7 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
@@ -4550,28 +4550,28 @@
         <v>118</v>
       </c>
       <c r="B13" s="4">
-        <v>22.406214182780552</v>
+        <v>5.8959533777770433E-2</v>
       </c>
       <c r="C13" s="4">
-        <v>22.431484487702846</v>
+        <v>0.44510460129921381</v>
       </c>
       <c r="D13" s="4">
-        <v>23.029835391621909</v>
+        <v>1.5082115649955179</v>
       </c>
       <c r="E13" s="4">
-        <v>23.699761446752497</v>
+        <v>1.6037486744545419</v>
       </c>
       <c r="F13" s="4">
-        <v>23.239570607204612</v>
+        <v>1.436164357778579</v>
       </c>
       <c r="G13" s="4">
-        <v>23.11169281392214</v>
+        <v>1.414182314808202</v>
       </c>
       <c r="H13" s="4">
-        <v>23.651461345313169</v>
+        <v>2.2996325762050698</v>
       </c>
       <c r="I13" s="4">
-        <v>24.328718542325902</v>
+        <v>2.324895408937842</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
@@ -4579,28 +4579,28 @@
         <v>119</v>
       </c>
       <c r="B14" s="4">
-        <v>22.254033212241392</v>
+        <v>2.9096507323751242E-2</v>
       </c>
       <c r="C14" s="4">
-        <v>22.347517640209603</v>
+        <v>0.49352969837321831</v>
       </c>
       <c r="D14" s="4">
-        <v>22.870934661486103</v>
+        <v>1.544857795446775</v>
       </c>
       <c r="E14" s="4">
-        <v>23.588050433340207</v>
+        <v>1.6830470454865321</v>
       </c>
       <c r="F14" s="4">
-        <v>23.167254457156844</v>
+        <v>1.373492108345697</v>
       </c>
       <c r="G14" s="4">
-        <v>22.963735902901391</v>
+        <v>1.518839232996644</v>
       </c>
       <c r="H14" s="4">
-        <v>23.52605909694401</v>
+        <v>2.2602503485082091</v>
       </c>
       <c r="I14" s="4">
-        <v>24.219364795765536</v>
+        <v>2.4084032241001738</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
@@ -4608,28 +4608,28 @@
         <v>120</v>
       </c>
       <c r="B15" s="4">
-        <v>81.44858461940494</v>
+        <v>2.2318106722052482</v>
       </c>
       <c r="C15" s="4">
-        <v>81.765178707868472</v>
+        <v>1.6505060810864389</v>
       </c>
       <c r="D15" s="4">
-        <v>81.660582435762095</v>
+        <v>2.942633574853279</v>
       </c>
       <c r="E15" s="4">
-        <v>84.368804010041757</v>
+        <v>3.4913373115757822</v>
       </c>
       <c r="F15" s="4">
-        <v>84.291794737675957</v>
+        <v>3.8608459040129661</v>
       </c>
       <c r="G15" s="4">
-        <v>82.209078553834615</v>
+        <v>3.2759752917558398</v>
       </c>
       <c r="H15" s="4">
-        <v>81.921717965610796</v>
+        <v>3.961105010967362</v>
       </c>
       <c r="I15" s="4">
-        <v>85.340090281800656</v>
+        <v>4.4634382492894744</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
@@ -4637,28 +4637,28 @@
         <v>121</v>
       </c>
       <c r="B16" s="4">
-        <v>81.449508079029769</v>
+        <v>0.35566838133519629</v>
       </c>
       <c r="C16" s="4">
-        <v>81.764999756290763</v>
+        <v>1.6478039201613519</v>
       </c>
       <c r="D16" s="4">
-        <v>81.661071364950246</v>
+        <v>3.041561602062977</v>
       </c>
       <c r="E16" s="4">
-        <v>84.369097680632564</v>
+        <v>3.4635888692955779</v>
       </c>
       <c r="F16" s="4">
-        <v>84.286671628156</v>
+        <v>3.4339602144278611</v>
       </c>
       <c r="G16" s="4">
-        <v>82.208054181133519</v>
+        <v>3.7504411444848351</v>
       </c>
       <c r="H16" s="4">
-        <v>81.919826361842482</v>
+        <v>3.9846117540619339</v>
       </c>
       <c r="I16" s="4">
-        <v>85.341039203421943</v>
+        <v>4.3938329698888214</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
version 3 cleaned up: tests green, add tools package and validation stub, pytest.ini
</commit_message>
<xml_diff>
--- a/Distributions/sensitivity_run_results_25012026.xlsx
+++ b/Distributions/sensitivity_run_results_25012026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://esait-my.sharepoint.com/personal/ivo_ferreira_esa_int/Documents/NewAthenaE2EPSF_v3/Distributions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="150" documentId="8_{E1C7CD1F-9ABC-5249-9B87-D7756653E306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10D268E6-8F7F-D14F-BE36-E381604D2AD4}"/>
+  <xr:revisionPtr revIDLastSave="152" documentId="8_{E1C7CD1F-9ABC-5249-9B87-D7756653E306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{06405731-9200-E64E-BD83-30C61D97B5D6}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2874,8 +2874,8 @@
     </pivotField>
     <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
       <items count="3">
-        <item x="0"/>
-        <item h="1" x="1"/>
+        <item h="1" x="0"/>
+        <item x="1"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -4462,7 +4462,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
@@ -4550,28 +4550,28 @@
         <v>118</v>
       </c>
       <c r="B13" s="4">
-        <v>5.8959533777770433E-2</v>
+        <v>8.0164876257149942</v>
       </c>
       <c r="C13" s="4">
-        <v>0.44510460129921381</v>
+        <v>8.0252594735309177</v>
       </c>
       <c r="D13" s="4">
-        <v>1.5082115649955179</v>
+        <v>8.2049513848246605</v>
       </c>
       <c r="E13" s="4">
-        <v>1.6037486744545419</v>
+        <v>8.2770170146274111</v>
       </c>
       <c r="F13" s="4">
-        <v>1.436164357778579</v>
+        <v>8.182731560501157</v>
       </c>
       <c r="G13" s="4">
-        <v>1.414182314808202</v>
+        <v>8.220820187647222</v>
       </c>
       <c r="H13" s="4">
-        <v>2.2996325762050698</v>
+        <v>8.3180344880370836</v>
       </c>
       <c r="I13" s="4">
-        <v>2.324895408937842</v>
+        <v>8.4651277177990352</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
@@ -4579,28 +4579,28 @@
         <v>119</v>
       </c>
       <c r="B14" s="4">
-        <v>2.9096507323751242E-2</v>
+        <v>7.9232585706283043</v>
       </c>
       <c r="C14" s="4">
-        <v>0.49352969837321831</v>
+        <v>7.9413138002692962</v>
       </c>
       <c r="D14" s="4">
-        <v>1.544857795446775</v>
+        <v>8.1421474065148143</v>
       </c>
       <c r="E14" s="4">
-        <v>1.6830470454865321</v>
+        <v>8.1886536292386349</v>
       </c>
       <c r="F14" s="4">
-        <v>1.373492108345697</v>
+        <v>8.123159315563063</v>
       </c>
       <c r="G14" s="4">
-        <v>1.518839232996644</v>
+        <v>8.155639757920552</v>
       </c>
       <c r="H14" s="4">
-        <v>2.2602503485082091</v>
+        <v>8.3516723562663984</v>
       </c>
       <c r="I14" s="4">
-        <v>2.4084032241001738</v>
+        <v>8.4016433536032284</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
@@ -4608,28 +4608,28 @@
         <v>120</v>
       </c>
       <c r="B15" s="4">
-        <v>2.2318106722052482</v>
+        <v>25.473639146600821</v>
       </c>
       <c r="C15" s="4">
-        <v>1.6505060810864389</v>
+        <v>25.47377529106916</v>
       </c>
       <c r="D15" s="4">
-        <v>2.942633574853279</v>
+        <v>26.08565449324831</v>
       </c>
       <c r="E15" s="4">
-        <v>3.4913373115757822</v>
+        <v>25.622668798625039</v>
       </c>
       <c r="F15" s="4">
-        <v>3.8608459040129661</v>
+        <v>26.135765115571601</v>
       </c>
       <c r="G15" s="4">
-        <v>3.2759752917558398</v>
+        <v>26.080696034291201</v>
       </c>
       <c r="H15" s="4">
-        <v>3.961105010967362</v>
+        <v>27.148993917077409</v>
       </c>
       <c r="I15" s="4">
-        <v>4.4634382492894744</v>
+        <v>26.213626397030371</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
@@ -4637,28 +4637,28 @@
         <v>121</v>
       </c>
       <c r="B16" s="4">
-        <v>0.35566838133519629</v>
+        <v>25.470102965834339</v>
       </c>
       <c r="C16" s="4">
-        <v>1.6478039201613519</v>
+        <v>25.48039237974718</v>
       </c>
       <c r="D16" s="4">
-        <v>3.041561602062977</v>
+        <v>26.075599104352921</v>
       </c>
       <c r="E16" s="4">
-        <v>3.4635888692955779</v>
+        <v>25.62387391908603</v>
       </c>
       <c r="F16" s="4">
-        <v>3.4339602144278611</v>
+        <v>26.13379376712302</v>
       </c>
       <c r="G16" s="4">
-        <v>3.7504411444848351</v>
+        <v>26.081000197336149</v>
       </c>
       <c r="H16" s="4">
-        <v>3.9846117540619339</v>
+        <v>27.126030815124349</v>
       </c>
       <c r="I16" s="4">
-        <v>4.3938329698888214</v>
+        <v>26.217027949117099</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added preliminary implementation to export fits file of the PSF and a csv file of the EEF graph
</commit_message>
<xml_diff>
--- a/Distributions/sensitivity_run_results_25012026.xlsx
+++ b/Distributions/sensitivity_run_results_25012026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://esait-my.sharepoint.com/personal/ivo_ferreira_esa_int/Documents/NewAthenaE2EPSF_v3/Distributions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="152" documentId="8_{E1C7CD1F-9ABC-5249-9B87-D7756653E306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{06405731-9200-E64E-BD83-30C61D97B5D6}"/>
+  <xr:revisionPtr revIDLastSave="156" documentId="8_{E1C7CD1F-9ABC-5249-9B87-D7756653E306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ED842AB5-C83F-294E-AFAA-3F5012C5356A}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="68800" windowHeight="26880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="801" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="801" uniqueCount="125">
   <si>
     <t>combo_id</t>
   </si>
@@ -409,6 +409,9 @@
   </si>
   <si>
     <t>Values</t>
+  </si>
+  <si>
+    <t>(Multiple Items)</t>
   </si>
 </sst>
 </file>
@@ -2888,17 +2891,17 @@
     </pivotField>
     <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
       <items count="3">
-        <item x="0"/>
-        <item h="1" x="1"/>
+        <item h="1" x="0"/>
+        <item x="1"/>
         <item t="default"/>
       </items>
     </pivotField>
-    <pivotField axis="axisPage" showAll="0">
+    <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
       <items count="5">
         <item x="0"/>
         <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
+        <item h="1" x="2"/>
+        <item h="1" x="3"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -3801,7 +3804,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
@@ -4470,7 +4473,7 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>23</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
@@ -4478,7 +4481,7 @@
         <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
@@ -4550,28 +4553,28 @@
         <v>118</v>
       </c>
       <c r="B13" s="4">
-        <v>8.0164876257149942</v>
+        <v>7.9723483070177448</v>
       </c>
       <c r="C13" s="4">
-        <v>8.0252594735309177</v>
+        <v>8.0870626122534865</v>
       </c>
       <c r="D13" s="4">
-        <v>8.2049513848246605</v>
+        <v>8.1086044945096685</v>
       </c>
       <c r="E13" s="4">
-        <v>8.2770170146274111</v>
+        <v>8.2713987172055479</v>
       </c>
       <c r="F13" s="4">
-        <v>8.182731560501157</v>
+        <v>8.041151010614815</v>
       </c>
       <c r="G13" s="4">
-        <v>8.220820187647222</v>
+        <v>8.133039788271951</v>
       </c>
       <c r="H13" s="4">
-        <v>8.3180344880370836</v>
+        <v>8.3915634693586085</v>
       </c>
       <c r="I13" s="4">
-        <v>8.4651277177990352</v>
+        <v>8.4183432329207388</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
@@ -4579,28 +4582,28 @@
         <v>119</v>
       </c>
       <c r="B14" s="4">
-        <v>7.9232585706283043</v>
+        <v>7.8923100631508092</v>
       </c>
       <c r="C14" s="4">
-        <v>7.9413138002692962</v>
+        <v>8.0490706066181108</v>
       </c>
       <c r="D14" s="4">
-        <v>8.1421474065148143</v>
+        <v>8.010478112954603</v>
       </c>
       <c r="E14" s="4">
-        <v>8.1886536292386349</v>
+        <v>8.2086823139831697</v>
       </c>
       <c r="F14" s="4">
-        <v>8.123159315563063</v>
+        <v>8.026213348084859</v>
       </c>
       <c r="G14" s="4">
-        <v>8.155639757920552</v>
+        <v>8.0626537721583649</v>
       </c>
       <c r="H14" s="4">
-        <v>8.3516723562663984</v>
+        <v>8.326020822789209</v>
       </c>
       <c r="I14" s="4">
-        <v>8.4016433536032284</v>
+        <v>8.3523870366237674</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
@@ -4608,28 +4611,28 @@
         <v>120</v>
       </c>
       <c r="B15" s="4">
-        <v>25.473639146600821</v>
+        <v>26.007092592596901</v>
       </c>
       <c r="C15" s="4">
-        <v>25.47377529106916</v>
+        <v>26.999468371575158</v>
       </c>
       <c r="D15" s="4">
-        <v>26.08565449324831</v>
+        <v>25.606987210898879</v>
       </c>
       <c r="E15" s="4">
-        <v>25.622668798625039</v>
+        <v>26.417037970735951</v>
       </c>
       <c r="F15" s="4">
-        <v>26.135765115571601</v>
+        <v>26.474919662056489</v>
       </c>
       <c r="G15" s="4">
-        <v>26.080696034291201</v>
+        <v>26.01821133820906</v>
       </c>
       <c r="H15" s="4">
-        <v>27.148993917077409</v>
+        <v>26.78332061436257</v>
       </c>
       <c r="I15" s="4">
-        <v>26.213626397030371</v>
+        <v>26.518367489819148</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
@@ -4637,28 +4640,28 @@
         <v>121</v>
       </c>
       <c r="B16" s="4">
-        <v>25.470102965834339</v>
+        <v>26.00756507169574</v>
       </c>
       <c r="C16" s="4">
-        <v>25.48039237974718</v>
+        <v>26.99966952018789</v>
       </c>
       <c r="D16" s="4">
-        <v>26.075599104352921</v>
+        <v>25.607534295966911</v>
       </c>
       <c r="E16" s="4">
-        <v>25.62387391908603</v>
+        <v>26.417263595506071</v>
       </c>
       <c r="F16" s="4">
-        <v>26.13379376712302</v>
+        <v>26.474769199711989</v>
       </c>
       <c r="G16" s="4">
-        <v>26.081000197336149</v>
+        <v>26.018283738110451</v>
       </c>
       <c r="H16" s="4">
-        <v>27.126030815124349</v>
+        <v>26.783161618254908</v>
       </c>
       <c r="I16" s="4">
-        <v>26.217027949117099</v>
+        <v>26.518816870867479</v>
       </c>
     </row>
   </sheetData>

</xml_diff>